<commit_message>
Collected code for submission
</commit_message>
<xml_diff>
--- a/1EMEsubmission_RasmusKristofferPedersen.xlsx
+++ b/1EMEsubmission_RasmusKristofferPedersen.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedersen\Documents\Research\1EME\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedersen\Documents\Github\1EME\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22EBCB70-574C-48B8-A72E-2C917C221C16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F2A3ED0D-6A90-4E3C-AFB4-F94EBA268CA3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F2A3ED0D-6A90-4E3C-AFB4-F94EBA268CA3}"/>
   </bookViews>
   <sheets>
     <sheet name="Estimates 1 (total by state)" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,6 @@
     <sheet name="Estimates 6 (MD race)" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -543,7 +542,7 @@
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000000"/>
-    <numFmt numFmtId="170" formatCode="0.0000000"/>
+    <numFmt numFmtId="166" formatCode="0.0000000"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -598,7 +597,7 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>